<commit_message>
Update Interface RDM for a test
</commit_message>
<xml_diff>
--- a/src/Interface_RDM.xlsx
+++ b/src/Interface_RDM.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ClimateLeadGroup\Desktop\CLG_repositories\osemosys-rdm\src\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\josea\OneDrive\Desktop\CLG_tests\osemosys-rdm\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD3D6553-1366-410F-9243-BC75801B889E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B8E30F1-BE8F-48D4-A9FF-89192E9D3801}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="727" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="727" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Uncertainty_Table" sheetId="1" r:id="rId1"/>
@@ -697,7 +697,7 @@
     <t>YES</t>
   </si>
   <si>
-    <t>cplex</t>
+    <t>cbc</t>
   </si>
 </sst>
 </file>
@@ -2060,7 +2060,7 @@
     </row>
     <row r="2" spans="1:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>74</v>
@@ -2069,7 +2069,7 @@
         <v>1</v>
       </c>
       <c r="D2" s="8">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="E2" s="9">
         <v>8</v>

</xml_diff>

<commit_message>
Update Interface RDM for a test with 100 futures and cplex solver
</commit_message>
<xml_diff>
--- a/src/Interface_RDM.xlsx
+++ b/src/Interface_RDM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\josea\OneDrive\Desktop\CLG_tests\osemosys-rdm\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B8E30F1-BE8F-48D4-A9FF-89192E9D3801}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FD1A41C-F93C-4613-A4D7-5AD7483126FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="727" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -697,7 +697,7 @@
     <t>YES</t>
   </si>
   <si>
-    <t>cbc</t>
+    <t>cplex</t>
   </si>
 </sst>
 </file>
@@ -2060,7 +2060,7 @@
     </row>
     <row r="2" spans="1:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
-        <v>4</v>
+        <v>100</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>74</v>
@@ -2069,7 +2069,7 @@
         <v>1</v>
       </c>
       <c r="D2" s="8">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="E2" s="9">
         <v>8</v>

</xml_diff>

<commit_message>
update scenario names in Interface_RDM and update Scenario.txt with Uganda model
</commit_message>
<xml_diff>
--- a/src/Interface_RDM.xlsx
+++ b/src/Interface_RDM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ClimateLeadGroup\Desktop\CLG_repositories\osemosys-rdm\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{457CAC94-DD2F-41D3-8231-F1F712EB66B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5FB203F-281F-4C12-887B-1100501FEE33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="727" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="727" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Uncertainty_Table" sheetId="1" r:id="rId1"/>
@@ -104,7 +104,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="193">
   <si>
     <t>Number_of_Runs</t>
   </si>
@@ -681,6 +681,9 @@
   </si>
   <si>
     <t>cplex</t>
+  </si>
+  <si>
+    <t>Scenario1</t>
   </si>
 </sst>
 </file>
@@ -1466,7 +1469,7 @@
         <v>38</v>
       </c>
       <c r="D2" s="25" t="s">
-        <v>39</v>
+        <v>192</v>
       </c>
       <c r="E2" s="25" t="s">
         <v>40</v>
@@ -1516,7 +1519,7 @@
         <v>48</v>
       </c>
       <c r="D3" s="25" t="s">
-        <v>39</v>
+        <v>192</v>
       </c>
       <c r="E3" s="25" t="s">
         <v>40</v>
@@ -1566,7 +1569,7 @@
         <v>52</v>
       </c>
       <c r="D4" s="25" t="s">
-        <v>39</v>
+        <v>192</v>
       </c>
       <c r="E4" s="25" t="s">
         <v>40</v>
@@ -1614,7 +1617,7 @@
         <v>56</v>
       </c>
       <c r="D5" s="25" t="s">
-        <v>39</v>
+        <v>192</v>
       </c>
       <c r="E5" s="25" t="s">
         <v>40</v>
@@ -1662,7 +1665,7 @@
         <v>60</v>
       </c>
       <c r="D6" s="25" t="s">
-        <v>39</v>
+        <v>192</v>
       </c>
       <c r="E6" s="25" t="s">
         <v>40</v>
@@ -1712,7 +1715,7 @@
         <v>63</v>
       </c>
       <c r="D7" s="25" t="s">
-        <v>39</v>
+        <v>192</v>
       </c>
       <c r="E7" s="25" t="s">
         <v>40</v>
@@ -1762,7 +1765,7 @@
         <v>64</v>
       </c>
       <c r="D8" s="25" t="s">
-        <v>39</v>
+        <v>192</v>
       </c>
       <c r="E8" s="25" t="s">
         <v>40</v>
@@ -1812,7 +1815,7 @@
         <v>66</v>
       </c>
       <c r="D9" s="32" t="s">
-        <v>39</v>
+        <v>192</v>
       </c>
       <c r="E9" s="32" t="s">
         <v>40</v>
@@ -1862,7 +1865,7 @@
         <v>68</v>
       </c>
       <c r="D10" s="32" t="s">
-        <v>39</v>
+        <v>192</v>
       </c>
       <c r="E10" s="32" t="s">
         <v>40</v>
@@ -1912,7 +1915,7 @@
         <v>71</v>
       </c>
       <c r="D11" s="32" t="s">
-        <v>39</v>
+        <v>192</v>
       </c>
       <c r="E11" s="32" t="s">
         <v>40</v>
@@ -1962,7 +1965,7 @@
         <v>74</v>
       </c>
       <c r="D12" s="32" t="s">
-        <v>39</v>
+        <v>192</v>
       </c>
       <c r="E12" s="32" t="s">
         <v>40</v>
@@ -2012,7 +2015,7 @@
         <v>78</v>
       </c>
       <c r="D13" s="32" t="s">
-        <v>39</v>
+        <v>192</v>
       </c>
       <c r="E13" s="32" t="s">
         <v>40</v>
@@ -2062,7 +2065,7 @@
         <v>80</v>
       </c>
       <c r="D14" s="32" t="s">
-        <v>39</v>
+        <v>192</v>
       </c>
       <c r="E14" s="32" t="s">
         <v>40</v>
@@ -2112,7 +2115,7 @@
         <v>83</v>
       </c>
       <c r="D15" s="32" t="s">
-        <v>39</v>
+        <v>192</v>
       </c>
       <c r="E15" s="32" t="s">
         <v>40</v>

</xml_diff>

<commit_message>
Upgrade modelo form 5.0 to 5.3
</commit_message>
<xml_diff>
--- a/src/Interface_RDM.xlsx
+++ b/src/Interface_RDM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ClimateLeadGroup\Desktop\CLG_repositories\osemosys-rdm\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5FB203F-281F-4C12-887B-1100501FEE33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D28DE246-1B5E-42F4-A0E0-CAA3A5E3615D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="727" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="727" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Uncertainty_Table" sheetId="1" r:id="rId1"/>
@@ -104,7 +104,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="192">
   <si>
     <t>Number_of_Runs</t>
   </si>
@@ -157,9 +157,6 @@
     <t>Yes</t>
   </si>
   <si>
-    <t>model.v.5.0.txt</t>
-  </si>
-  <si>
     <t>UGA</t>
   </si>
   <si>
@@ -221,9 +218,6 @@
   </si>
   <si>
     <t xml:space="preserve">Minimum share of solid waste that should be collected </t>
-  </si>
-  <si>
-    <t>BAU ; Scenario1</t>
   </si>
   <si>
     <t>Time_Series</t>
@@ -684,6 +678,9 @@
   </si>
   <si>
     <t>Scenario1</t>
+  </si>
+  <si>
+    <t>model.v.5.3.txt</t>
   </si>
 </sst>
 </file>
@@ -1404,58 +1401,58 @@
   <sheetData>
     <row r="1" spans="1:18" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="C1" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="D1" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="E1" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="E1" s="16" t="s">
+      <c r="F1" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="F1" s="16" t="s">
+      <c r="G1" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="G1" s="16" t="s">
+      <c r="H1" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="H1" s="16" t="s">
+      <c r="I1" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="I1" s="16" t="s">
+      <c r="J1" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="J1" s="16" t="s">
+      <c r="K1" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="18" t="s">
+      <c r="L1" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="L1" s="17" t="s">
+      <c r="M1" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="M1" s="17" t="s">
+      <c r="N1" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="N1" s="16" t="s">
+      <c r="O1" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="O1" s="17" t="s">
+      <c r="P1" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="P1" s="16" t="s">
+      <c r="Q1" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="Q1" s="16" t="s">
+      <c r="R1" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="R1" s="16" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -1463,19 +1460,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="25" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="C2" s="26" t="s">
+      <c r="D2" s="25" t="s">
+        <v>190</v>
+      </c>
+      <c r="E2" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="D2" s="25" t="s">
-        <v>192</v>
-      </c>
-      <c r="E2" s="25" t="s">
-        <v>40</v>
-      </c>
       <c r="F2" s="25" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G2" s="25">
         <v>2026</v>
@@ -1487,22 +1484,22 @@
         <v>1</v>
       </c>
       <c r="J2" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="K2" s="27" t="s">
+        <v>41</v>
+      </c>
+      <c r="L2" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="K2" s="27" t="s">
+      <c r="M2" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="L2" s="28" t="s">
+      <c r="N2" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="M2" s="26" t="s">
+      <c r="O2" s="26" t="s">
         <v>45</v>
-      </c>
-      <c r="N2" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="O2" s="26" t="s">
-        <v>47</v>
       </c>
       <c r="P2" s="25"/>
       <c r="Q2" s="25"/>
@@ -1513,19 +1510,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="25" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C3" s="26" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D3" s="25" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="E3" s="25" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F3" s="25" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G3" s="25">
         <v>2026</v>
@@ -1537,22 +1534,22 @@
         <v>1</v>
       </c>
       <c r="J3" s="25" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="K3" s="27" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="L3" s="29" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="M3" s="26" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="N3" s="26" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="O3" s="26" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="P3" s="25"/>
       <c r="Q3" s="25"/>
@@ -1563,19 +1560,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="26" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C4" s="26" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D4" s="25" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="E4" s="25" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F4" s="25" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G4" s="25">
         <v>2026</v>
@@ -1587,20 +1584,20 @@
         <v>1.3</v>
       </c>
       <c r="J4" s="30" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="K4" s="27" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="L4" s="31" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="M4" s="29">
         <v>1</v>
       </c>
       <c r="N4" s="26"/>
       <c r="O4" s="26" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="P4" s="25"/>
       <c r="Q4" s="25"/>
@@ -1611,19 +1608,19 @@
         <v>4</v>
       </c>
       <c r="B5" s="26" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C5" s="26" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D5" s="25" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="E5" s="25" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F5" s="25" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G5" s="25">
         <v>2026</v>
@@ -1635,20 +1632,20 @@
         <v>1.4</v>
       </c>
       <c r="J5" s="30" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K5" s="27" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="L5" s="31" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="M5" s="29" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="N5" s="26"/>
       <c r="O5" s="26" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="P5" s="25"/>
       <c r="Q5" s="25"/>
@@ -1659,19 +1656,19 @@
         <v>5</v>
       </c>
       <c r="B6" s="26" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C6" s="26" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D6" s="25" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="E6" s="25" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F6" s="25" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G6" s="25">
         <v>2026</v>
@@ -1683,22 +1680,22 @@
         <v>1.4</v>
       </c>
       <c r="J6" s="30" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="K6" s="27" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="L6" s="29" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M6" s="29" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="N6" s="26" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="O6" s="26" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="P6" s="25"/>
       <c r="Q6" s="25"/>
@@ -1709,19 +1706,19 @@
         <v>6</v>
       </c>
       <c r="B7" s="26" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C7" s="26" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D7" s="25" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="E7" s="25" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F7" s="25" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G7" s="25">
         <v>2026</v>
@@ -1733,22 +1730,22 @@
         <v>1.2</v>
       </c>
       <c r="J7" s="30" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K7" s="27" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="L7" s="29" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M7" s="29" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="N7" s="26" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="O7" s="26" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="P7" s="25"/>
       <c r="Q7" s="25"/>
@@ -1759,19 +1756,19 @@
         <v>7</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C8" s="26" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D8" s="25" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="E8" s="25" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F8" s="25" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G8" s="25">
         <v>2026</v>
@@ -1783,22 +1780,22 @@
         <v>1.2</v>
       </c>
       <c r="J8" s="30" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="K8" s="27" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="L8" s="29" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="M8" s="29" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="N8" s="26" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="O8" s="26" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="P8" s="25"/>
       <c r="Q8" s="25"/>
@@ -1809,19 +1806,19 @@
         <v>8</v>
       </c>
       <c r="B9" s="32" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C9" s="34" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D9" s="32" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="E9" s="32" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F9" s="32" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G9" s="32">
         <v>2026</v>
@@ -1833,22 +1830,22 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="J9" s="32" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K9" s="33" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="L9" s="35" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="M9" s="34" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="N9" s="34" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="O9" s="34" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="P9" s="32"/>
       <c r="Q9" s="32"/>
@@ -1859,19 +1856,19 @@
         <v>9</v>
       </c>
       <c r="B10" s="32" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C10" s="34" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D10" s="32" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="E10" s="32" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F10" s="32" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G10" s="32">
         <v>2026</v>
@@ -1883,22 +1880,22 @@
         <v>1.2</v>
       </c>
       <c r="J10" s="32" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K10" s="33" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="L10" s="35" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="M10" s="34" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="N10" s="34" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="O10" s="34" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="P10" s="32"/>
       <c r="Q10" s="32"/>
@@ -1909,19 +1906,19 @@
         <v>10</v>
       </c>
       <c r="B11" s="32" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C11" s="34" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D11" s="32" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="E11" s="32" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F11" s="32" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G11" s="32">
         <v>2026</v>
@@ -1933,22 +1930,22 @@
         <v>1.5</v>
       </c>
       <c r="J11" s="32" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="K11" s="33" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="L11" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="M11" s="32">
         <v>1</v>
       </c>
       <c r="N11" s="34" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="O11" s="34" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="P11" s="32"/>
       <c r="Q11" s="32"/>
@@ -1959,19 +1956,19 @@
         <v>11</v>
       </c>
       <c r="B12" s="32" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C12" s="34" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D12" s="32" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="E12" s="32" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F12" s="32" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G12" s="32">
         <v>2026</v>
@@ -1983,22 +1980,22 @@
         <v>1.2</v>
       </c>
       <c r="J12" s="32" t="s">
+        <v>73</v>
+      </c>
+      <c r="K12" s="33" t="s">
+        <v>41</v>
+      </c>
+      <c r="L12" s="35" t="s">
+        <v>74</v>
+      </c>
+      <c r="M12" s="34" t="s">
         <v>75</v>
       </c>
-      <c r="K12" s="33" t="s">
-        <v>43</v>
-      </c>
-      <c r="L12" s="35" t="s">
-        <v>76</v>
-      </c>
-      <c r="M12" s="34" t="s">
-        <v>77</v>
-      </c>
       <c r="N12" s="34">
         <v>1</v>
       </c>
       <c r="O12" s="34" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="P12" s="32"/>
       <c r="Q12" s="32"/>
@@ -2009,19 +2006,19 @@
         <v>12</v>
       </c>
       <c r="B13" s="32" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C13" s="34" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D13" s="32" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="E13" s="32" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F13" s="32" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G13" s="32">
         <v>2026</v>
@@ -2033,22 +2030,22 @@
         <v>1.5</v>
       </c>
       <c r="J13" s="32" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="K13" s="33" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="L13" s="35" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="M13" s="34" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="N13" s="34" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="O13" s="34" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="P13" s="32"/>
       <c r="Q13" s="32"/>
@@ -2059,19 +2056,19 @@
         <v>13</v>
       </c>
       <c r="B14" s="32" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C14" s="32" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D14" s="32" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="E14" s="32" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F14" s="32" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G14" s="32">
         <v>2026</v>
@@ -2083,22 +2080,22 @@
         <v>1.3</v>
       </c>
       <c r="J14" s="32" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="K14" s="33" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="L14" s="34" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="M14" s="34" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="N14" s="32" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="O14" s="34" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="P14" s="32"/>
       <c r="Q14" s="32"/>
@@ -2109,19 +2106,19 @@
         <v>14</v>
       </c>
       <c r="B15" s="32" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C15" s="32" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D15" s="32" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="E15" s="32" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F15" s="32" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G15" s="32">
         <v>2026</v>
@@ -2133,22 +2130,22 @@
         <v>1.2</v>
       </c>
       <c r="J15" s="32" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="K15" s="33" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="L15" s="34" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="M15" s="34" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="N15" s="34">
         <v>1</v>
       </c>
       <c r="O15" s="34" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="P15" s="32"/>
       <c r="Q15" s="32"/>
@@ -3415,13 +3412,13 @@
         <v>16</v>
       </c>
       <c r="H2" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="I2" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="J2" s="13" t="s">
         <v>17</v>
-      </c>
-      <c r="J2" s="13" t="s">
-        <v>18</v>
       </c>
       <c r="K2" s="13"/>
       <c r="L2" s="13"/>
@@ -3445,186 +3442,186 @@
   <sheetData>
     <row r="1" spans="1:59" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C1" t="s">
         <v>86</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>87</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>88</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>89</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>90</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>91</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>92</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>93</v>
       </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>94</v>
       </c>
-      <c r="J1" t="s">
+      <c r="L1" t="s">
         <v>95</v>
       </c>
-      <c r="K1" t="s">
+      <c r="M1" t="s">
         <v>96</v>
       </c>
-      <c r="L1" t="s">
+      <c r="N1" t="s">
+        <v>67</v>
+      </c>
+      <c r="O1" t="s">
         <v>97</v>
       </c>
-      <c r="M1" t="s">
+      <c r="P1" t="s">
         <v>98</v>
       </c>
-      <c r="N1" t="s">
-        <v>69</v>
-      </c>
-      <c r="O1" t="s">
+      <c r="Q1" t="s">
         <v>99</v>
       </c>
-      <c r="P1" t="s">
+      <c r="R1" t="s">
         <v>100</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="S1" t="s">
         <v>101</v>
       </c>
-      <c r="R1" t="s">
+      <c r="T1" t="s">
         <v>102</v>
       </c>
-      <c r="S1" t="s">
+      <c r="U1" t="s">
         <v>103</v>
       </c>
-      <c r="T1" t="s">
+      <c r="V1" t="s">
+        <v>73</v>
+      </c>
+      <c r="W1" t="s">
         <v>104</v>
       </c>
-      <c r="U1" t="s">
+      <c r="X1" t="s">
         <v>105</v>
       </c>
-      <c r="V1" t="s">
-        <v>75</v>
-      </c>
-      <c r="W1" t="s">
+      <c r="Y1" t="s">
+        <v>82</v>
+      </c>
+      <c r="Z1" t="s">
         <v>106</v>
       </c>
-      <c r="X1" t="s">
+      <c r="AA1" t="s">
+        <v>59</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>51</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>55</v>
+      </c>
+      <c r="AD1" t="s">
         <v>107</v>
       </c>
-      <c r="Y1" t="s">
-        <v>84</v>
-      </c>
-      <c r="Z1" t="s">
+      <c r="AE1" t="s">
         <v>108</v>
       </c>
-      <c r="AA1" t="s">
-        <v>61</v>
-      </c>
-      <c r="AB1" t="s">
-        <v>53</v>
-      </c>
-      <c r="AC1" t="s">
-        <v>57</v>
-      </c>
-      <c r="AD1" t="s">
+      <c r="AF1" t="s">
         <v>109</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AG1" t="s">
         <v>110</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AH1" t="s">
         <v>111</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AI1" t="s">
         <v>112</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AJ1" t="s">
         <v>113</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AK1" t="s">
         <v>114</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AL1" t="s">
         <v>115</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AM1" t="s">
         <v>116</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AN1" t="s">
         <v>117</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AO1" t="s">
         <v>118</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AP1" t="s">
         <v>119</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AQ1" t="s">
         <v>120</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AR1" t="s">
         <v>121</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="AS1" t="s">
         <v>122</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AT1" t="s">
         <v>123</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="AU1" t="s">
         <v>124</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="AV1" t="s">
         <v>125</v>
       </c>
-      <c r="AU1" t="s">
+      <c r="AW1" t="s">
+        <v>107</v>
+      </c>
+      <c r="AX1" t="s">
         <v>126</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="AY1" t="s">
         <v>127</v>
       </c>
-      <c r="AW1" t="s">
-        <v>109</v>
-      </c>
-      <c r="AX1" t="s">
+      <c r="AZ1" t="s">
         <v>128</v>
       </c>
-      <c r="AY1" t="s">
+      <c r="BA1" t="s">
         <v>129</v>
       </c>
-      <c r="AZ1" t="s">
+      <c r="BB1" t="s">
         <v>130</v>
       </c>
-      <c r="BA1" t="s">
+      <c r="BC1" t="s">
         <v>131</v>
       </c>
-      <c r="BB1" t="s">
+      <c r="BD1" t="s">
+        <v>40</v>
+      </c>
+      <c r="BE1" t="s">
         <v>132</v>
       </c>
-      <c r="BC1" t="s">
+      <c r="BF1" t="s">
         <v>133</v>
       </c>
-      <c r="BD1" t="s">
-        <v>42</v>
-      </c>
-      <c r="BE1" t="s">
+      <c r="BG1" t="s">
         <v>134</v>
-      </c>
-      <c r="BF1" t="s">
-        <v>135</v>
-      </c>
-      <c r="BG1" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="2" spans="1:59" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -3803,260 +3800,260 @@
     </row>
     <row r="3" spans="1:59" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
+        <v>136</v>
+      </c>
+      <c r="C3" t="s">
+        <v>137</v>
+      </c>
+      <c r="D3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E3" t="s">
+        <v>137</v>
+      </c>
+      <c r="F3" t="s">
+        <v>137</v>
+      </c>
+      <c r="G3" t="s">
+        <v>136</v>
+      </c>
+      <c r="H3" t="s">
+        <v>136</v>
+      </c>
+      <c r="I3" t="s">
+        <v>136</v>
+      </c>
+      <c r="J3" t="s">
         <v>138</v>
       </c>
-      <c r="C3" t="s">
+      <c r="K3" t="s">
         <v>139</v>
       </c>
-      <c r="D3" t="s">
-        <v>139</v>
-      </c>
-      <c r="E3" t="s">
-        <v>139</v>
-      </c>
-      <c r="F3" t="s">
-        <v>139</v>
-      </c>
-      <c r="G3" t="s">
-        <v>138</v>
-      </c>
-      <c r="H3" t="s">
-        <v>138</v>
-      </c>
-      <c r="I3" t="s">
-        <v>138</v>
-      </c>
-      <c r="J3" t="s">
+      <c r="L3" t="s">
         <v>140</v>
       </c>
-      <c r="K3" t="s">
+      <c r="M3" t="s">
+        <v>140</v>
+      </c>
+      <c r="N3" t="s">
+        <v>140</v>
+      </c>
+      <c r="O3" t="s">
+        <v>137</v>
+      </c>
+      <c r="P3" t="s">
+        <v>137</v>
+      </c>
+      <c r="Q3" t="s">
         <v>141</v>
       </c>
-      <c r="L3" t="s">
+      <c r="R3" t="s">
+        <v>141</v>
+      </c>
+      <c r="S3" t="s">
+        <v>141</v>
+      </c>
+      <c r="T3" t="s">
+        <v>137</v>
+      </c>
+      <c r="U3" t="s">
+        <v>141</v>
+      </c>
+      <c r="V3" t="s">
+        <v>141</v>
+      </c>
+      <c r="W3" t="s">
+        <v>141</v>
+      </c>
+      <c r="X3" t="s">
+        <v>141</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>141</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>137</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>141</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>141</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>141</v>
+      </c>
+      <c r="AD3" t="s">
         <v>142</v>
       </c>
-      <c r="M3" t="s">
+      <c r="AE3" t="s">
+        <v>141</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>141</v>
+      </c>
+      <c r="AG3" t="s">
+        <v>141</v>
+      </c>
+      <c r="AH3" t="s">
+        <v>141</v>
+      </c>
+      <c r="AI3" t="s">
+        <v>141</v>
+      </c>
+      <c r="AJ3" t="s">
+        <v>141</v>
+      </c>
+      <c r="AK3" t="s">
+        <v>141</v>
+      </c>
+      <c r="AL3" t="s">
+        <v>141</v>
+      </c>
+      <c r="AM3" t="s">
+        <v>141</v>
+      </c>
+      <c r="AN3" t="s">
+        <v>143</v>
+      </c>
+      <c r="AO3" t="s">
+        <v>143</v>
+      </c>
+      <c r="AP3" t="s">
+        <v>143</v>
+      </c>
+      <c r="AQ3" t="s">
+        <v>141</v>
+      </c>
+      <c r="AR3" t="s">
+        <v>141</v>
+      </c>
+      <c r="AS3" t="s">
+        <v>141</v>
+      </c>
+      <c r="AT3" t="s">
         <v>142</v>
       </c>
-      <c r="N3" t="s">
+      <c r="AU3" t="s">
         <v>142</v>
       </c>
-      <c r="O3" t="s">
-        <v>139</v>
-      </c>
-      <c r="P3" t="s">
-        <v>139</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>143</v>
-      </c>
-      <c r="R3" t="s">
-        <v>143</v>
-      </c>
-      <c r="S3" t="s">
-        <v>143</v>
-      </c>
-      <c r="T3" t="s">
-        <v>139</v>
-      </c>
-      <c r="U3" t="s">
-        <v>143</v>
-      </c>
-      <c r="V3" t="s">
-        <v>143</v>
-      </c>
-      <c r="W3" t="s">
-        <v>143</v>
-      </c>
-      <c r="X3" t="s">
-        <v>143</v>
-      </c>
-      <c r="Y3" t="s">
-        <v>143</v>
-      </c>
-      <c r="Z3" t="s">
-        <v>139</v>
-      </c>
-      <c r="AA3" t="s">
-        <v>143</v>
-      </c>
-      <c r="AB3" t="s">
-        <v>143</v>
-      </c>
-      <c r="AC3" t="s">
-        <v>143</v>
-      </c>
-      <c r="AD3" t="s">
+      <c r="AV3" t="s">
+        <v>137</v>
+      </c>
+      <c r="AW3" t="s">
+        <v>142</v>
+      </c>
+      <c r="AX3" t="s">
+        <v>142</v>
+      </c>
+      <c r="AY3" t="s">
+        <v>141</v>
+      </c>
+      <c r="AZ3" t="s">
+        <v>141</v>
+      </c>
+      <c r="BA3" t="s">
+        <v>141</v>
+      </c>
+      <c r="BB3" t="s">
+        <v>141</v>
+      </c>
+      <c r="BC3" t="s">
         <v>144</v>
       </c>
-      <c r="AE3" t="s">
-        <v>143</v>
-      </c>
-      <c r="AF3" t="s">
-        <v>143</v>
-      </c>
-      <c r="AG3" t="s">
-        <v>143</v>
-      </c>
-      <c r="AH3" t="s">
-        <v>143</v>
-      </c>
-      <c r="AI3" t="s">
-        <v>143</v>
-      </c>
-      <c r="AJ3" t="s">
-        <v>143</v>
-      </c>
-      <c r="AK3" t="s">
-        <v>143</v>
-      </c>
-      <c r="AL3" t="s">
-        <v>143</v>
-      </c>
-      <c r="AM3" t="s">
-        <v>143</v>
-      </c>
-      <c r="AN3" t="s">
-        <v>145</v>
-      </c>
-      <c r="AO3" t="s">
-        <v>145</v>
-      </c>
-      <c r="AP3" t="s">
-        <v>145</v>
-      </c>
-      <c r="AQ3" t="s">
-        <v>143</v>
-      </c>
-      <c r="AR3" t="s">
-        <v>143</v>
-      </c>
-      <c r="AS3" t="s">
-        <v>143</v>
-      </c>
-      <c r="AT3" t="s">
-        <v>144</v>
-      </c>
-      <c r="AU3" t="s">
-        <v>144</v>
-      </c>
-      <c r="AV3" t="s">
-        <v>139</v>
-      </c>
-      <c r="AW3" t="s">
-        <v>144</v>
-      </c>
-      <c r="AX3" t="s">
-        <v>144</v>
-      </c>
-      <c r="AY3" t="s">
-        <v>143</v>
-      </c>
-      <c r="AZ3" t="s">
-        <v>143</v>
-      </c>
-      <c r="BA3" t="s">
-        <v>143</v>
-      </c>
-      <c r="BB3" t="s">
-        <v>143</v>
-      </c>
-      <c r="BC3" t="s">
-        <v>146</v>
-      </c>
       <c r="BD3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="BE3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="BF3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="BG3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="4" spans="1:59" x14ac:dyDescent="0.3">
       <c r="M4" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="R4" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="V4" t="s">
+        <v>140</v>
+      </c>
+      <c r="W4" t="s">
+        <v>140</v>
+      </c>
+      <c r="X4" t="s">
+        <v>140</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>140</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>145</v>
+      </c>
+      <c r="AM4" t="s">
+        <v>143</v>
+      </c>
+      <c r="AQ4" t="s">
+        <v>143</v>
+      </c>
+      <c r="AR4" t="s">
         <v>142</v>
       </c>
-      <c r="W4" t="s">
+      <c r="AS4" t="s">
         <v>142</v>
       </c>
-      <c r="X4" t="s">
+      <c r="AV4" t="s">
         <v>142</v>
       </c>
-      <c r="Y4" t="s">
-        <v>142</v>
-      </c>
-      <c r="AB4" t="s">
-        <v>147</v>
-      </c>
-      <c r="AM4" t="s">
+      <c r="AY4" t="s">
         <v>145</v>
       </c>
-      <c r="AQ4" t="s">
+      <c r="AZ4" t="s">
         <v>145</v>
       </c>
-      <c r="AR4" t="s">
+      <c r="BA4" t="s">
+        <v>145</v>
+      </c>
+      <c r="BB4" t="s">
+        <v>145</v>
+      </c>
+      <c r="BD4" t="s">
         <v>144</v>
       </c>
-      <c r="AS4" t="s">
+      <c r="BE4" t="s">
         <v>144</v>
       </c>
-      <c r="AV4" t="s">
+      <c r="BF4" t="s">
         <v>144</v>
       </c>
-      <c r="AY4" t="s">
-        <v>147</v>
-      </c>
-      <c r="AZ4" t="s">
-        <v>147</v>
-      </c>
-      <c r="BA4" t="s">
-        <v>147</v>
-      </c>
-      <c r="BB4" t="s">
-        <v>147</v>
-      </c>
-      <c r="BD4" t="s">
-        <v>146</v>
-      </c>
-      <c r="BE4" t="s">
-        <v>146</v>
-      </c>
-      <c r="BF4" t="s">
-        <v>146</v>
-      </c>
       <c r="BG4" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="5" spans="1:59" x14ac:dyDescent="0.3">
       <c r="V5" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="Y5" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="AM5" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="AQ5" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="AR5" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="AS5" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -4075,237 +4072,237 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B8" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bring Interface_RDM.xlsx and Scenario1.txt from south-africa
</commit_message>
<xml_diff>
--- a/src/Interface_RDM.xlsx
+++ b/src/Interface_RDM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ClimateLeadGroup\Desktop\CLG_repositories\osemosys-rdm\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D28DE246-1B5E-42F4-A0E0-CAA3A5E3615D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{033E2F10-8602-4FA2-9BC2-5E9DEDE696C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="727" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="727" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Uncertainty_Table" sheetId="1" r:id="rId1"/>
@@ -104,7 +104,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="198">
   <si>
     <t>Number_of_Runs</t>
   </si>
@@ -157,7 +157,13 @@
     <t>Yes</t>
   </si>
   <si>
-    <t>UGA</t>
+    <t>cbc</t>
+  </si>
+  <si>
+    <t>model.v.5.0.txt</t>
+  </si>
+  <si>
+    <t>RSA</t>
   </si>
   <si>
     <t>X_Num</t>
@@ -214,10 +220,13 @@
     <t>Sum_To_Value</t>
   </si>
   <si>
-    <t>Collection rate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Minimum share of solid waste that should be collected </t>
+    <t>Capital Cost</t>
+  </si>
+  <si>
+    <t>Capital cost for NUCLEAR</t>
+  </si>
+  <si>
+    <t>Scenario1</t>
   </si>
   <si>
     <t>Time_Series</t>
@@ -226,289 +235,306 @@
     <t>Final_Value</t>
   </si>
   <si>
+    <t>CapitalCost</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>RSA_POW_PP_NU_OLD ; RSA_POW_PP_NU ; RSA_POW_PP_NU_SMR</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>1) Multiply final value of time series by the Explored Parameter in each future and then interpolate. 2) Assign the modified parameter back.</t>
+  </si>
+  <si>
+    <t>Capital Cost of competing technologies</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> RSA_POW_PP_HYDR ; RSA_POW_PP_CSP ; RSA_POW_PP_PV_UT ; RSA_POW_PP_PV_DIST ; RSA_POW_PP_WIND ; RSA_POW_STO_BAT_OUT ; RSA_POW_STO_PHY_OUT</t>
+  </si>
+  <si>
+    <t>Fixed Cost</t>
+  </si>
+  <si>
+    <t>Fixed Cost of competing technologies</t>
+  </si>
+  <si>
+    <t>FixedCost</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> RSA_POW_PP_HYDR ; RSA_POW_PP_CSP ; RSA_POW_PP_PV_UT ; RSA_POW_PP_PV_DIST ; RSA_POW_PP_WIND </t>
+  </si>
+  <si>
+    <t>Variable Cost</t>
+  </si>
+  <si>
+    <t>Variable Cost of competing technologies</t>
+  </si>
+  <si>
+    <t>VariableCost</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> RSA_POW_PP_CSP ; RSA_FUEL_PRO_NG  </t>
+  </si>
+  <si>
+    <t>1 ; 2</t>
+  </si>
+  <si>
+    <t>Capital Cost of competing technologies  FOSSIL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RSA_POW_PP_COAL ; RSA_POW_PP_MMG ; RSA_POW_PP_PEAK </t>
+  </si>
+  <si>
+    <t>Fixed Cost of competing technologies   FOSSIL</t>
+  </si>
+  <si>
+    <t>Variable Cost of competing technologies   FOSSIL</t>
+  </si>
+  <si>
+    <t>RSA_FUEL_PRO_COAL ; RSA_POW_PP_COAL ; RSA_POW_PP_MMG ; RSA_POW_PP_PEAK ; RSA_FUEL_PRO_DSL</t>
+  </si>
+  <si>
+    <t>Reserve Margin</t>
+  </si>
+  <si>
+    <t>Minimum non-intermittent capacity  the system should have</t>
+  </si>
+  <si>
+    <t>UDCMultiplierTotalCapacity</t>
+  </si>
+  <si>
+    <t>RSA_POW_TD</t>
+  </si>
+  <si>
+    <t>RESMAR</t>
+  </si>
+  <si>
+    <t>Cost of Transimission grids</t>
+  </si>
+  <si>
+    <t>Capacity Factor</t>
+  </si>
+  <si>
+    <t>Factor of Capacities</t>
+  </si>
+  <si>
+    <t>CapacityFactor</t>
+  </si>
+  <si>
+    <t>RSA_POW_PP_HYDR</t>
+  </si>
+  <si>
+    <t>All</t>
+  </si>
+  <si>
+    <t>Input Activity Ratio</t>
+  </si>
+  <si>
+    <t>Activity Ratio of Inputs</t>
+  </si>
+  <si>
+    <t>InputActivityRatio</t>
+  </si>
+  <si>
+    <t>RSA_FUEL_COAL ; RSA_FUEL_NG ; RSA_FUEL_NG</t>
+  </si>
+  <si>
+    <t>Emission Activity Ratio</t>
+  </si>
+  <si>
+    <t>Penalty to Emissions</t>
+  </si>
+  <si>
+    <t>EmissionActivityRatio</t>
+  </si>
+  <si>
+    <t>RSA_FUEL_PRO_COAL</t>
+  </si>
+  <si>
+    <t>RSA_CO2</t>
+  </si>
+  <si>
+    <t>Emission Penalty</t>
+  </si>
+  <si>
+    <t>EmissionsPenalty</t>
+  </si>
+  <si>
+    <t>Demand Profile</t>
+  </si>
+  <si>
+    <t>Specified Demand Profile of technologies</t>
+  </si>
+  <si>
+    <t>Timeslices_Curve</t>
+  </si>
+  <si>
+    <t>Change_Curve</t>
+  </si>
+  <si>
+    <t>SpecifiedDemandProfile</t>
+  </si>
+  <si>
+    <t>RSA_POW_ELEF</t>
+  </si>
+  <si>
+    <t>1) Select a curve from "shape_of_demand.xlsx". 2) The curve of the selected timeslices in the column “CF_timeslices” is changed to the selected curve of “shape_of_demand.xlsx”.</t>
+  </si>
+  <si>
+    <t>Demand Growth</t>
+  </si>
+  <si>
+    <t>Changes in the demand magnitude</t>
+  </si>
+  <si>
+    <t>SpecifiedAnnualDemand</t>
+  </si>
+  <si>
+    <t>parameter</t>
+  </si>
+  <si>
+    <t>YearSplit</t>
+  </si>
+  <si>
+    <t>DiscountRate</t>
+  </si>
+  <si>
+    <t>DiscountRateIdv</t>
+  </si>
+  <si>
+    <t>TradeRoute</t>
+  </si>
+  <si>
+    <t>DepreciationMethod</t>
+  </si>
+  <si>
+    <t>Conversionls</t>
+  </si>
+  <si>
+    <t>Conversionld</t>
+  </si>
+  <si>
+    <t>Conversionlh</t>
+  </si>
+  <si>
+    <t>DaySplit</t>
+  </si>
+  <si>
+    <t>DaysInDayType</t>
+  </si>
+  <si>
+    <t>AccumulatedAnnualDemand</t>
+  </si>
+  <si>
+    <t>CapacityToActivityUnit</t>
+  </si>
+  <si>
+    <t>CapitalRecoveryFactor</t>
+  </si>
+  <si>
+    <t>CapacityOfOneTechnologyUnit</t>
+  </si>
+  <si>
+    <t>AvailabilityFactor</t>
+  </si>
+  <si>
+    <t>OperationalLife</t>
+  </si>
+  <si>
+    <t>ResidualCapacity</t>
+  </si>
+  <si>
+    <t>InputToNewCapacityRatio</t>
+  </si>
+  <si>
+    <t>InputToTotalCapacityRatio</t>
+  </si>
+  <si>
+    <t>OutputActivityRatio</t>
+  </si>
+  <si>
+    <t>PvAnnuity</t>
+  </si>
+  <si>
+    <t>CapitalCostStorage</t>
+  </si>
+  <si>
+    <t>TotalAnnualMaxCapacity</t>
+  </si>
+  <si>
+    <t>TotalAnnualMinCapacity</t>
+  </si>
+  <si>
+    <t>TotalAnnualMaxCapacityInvestment</t>
+  </si>
+  <si>
+    <t>TotalAnnualMinCapacityInvestment</t>
+  </si>
+  <si>
+    <t>TotalTechnologyAnnualActivityUpperLimit</t>
+  </si>
+  <si>
+    <t>TotalTechnologyAnnualActivityLowerLimit</t>
+  </si>
+  <si>
+    <t>TotalTechnologyModelPeriodActivityUpperLimit</t>
+  </si>
+  <si>
+    <t>TotalTechnologyModelPeriodActivityLowerLimit</t>
+  </si>
+  <si>
+    <t>AnnualEmissionLimit</t>
+  </si>
+  <si>
+    <t>ModelPeriodEmissionLimit</t>
+  </si>
+  <si>
+    <t>EmissionToActivityChangeRatio</t>
+  </si>
+  <si>
+    <t>TechnologyFromStorage</t>
+  </si>
+  <si>
+    <t>TechnologyToStorage</t>
+  </si>
+  <si>
+    <t>StorageLevelStart</t>
+  </si>
+  <si>
+    <t>MinStorageCharge</t>
+  </si>
+  <si>
+    <t>OperationalLifeStorage</t>
+  </si>
+  <si>
+    <t>ResidualStorageCapacity</t>
+  </si>
+  <si>
+    <t>TechnologyActivityIncreaseByModeLimit</t>
+  </si>
+  <si>
+    <t>TechnologyActivityDecreaseByModeLimit</t>
+  </si>
+  <si>
+    <t>TechnologyActivityByModeLowerLimit</t>
+  </si>
+  <si>
+    <t>TechnologyActivityByModeUpperLimit</t>
+  </si>
+  <si>
+    <t>UDCConstant</t>
+  </si>
+  <si>
     <t>UDCMultiplierActivity</t>
   </si>
   <si>
-    <t>NO</t>
-  </si>
-  <si>
-    <t>WSTGEN</t>
-  </si>
-  <si>
-    <t>COLWST</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>1) Multiply final value of time series by the Explored Parameter in each future and then interpolate. 2) Assign the modified parameter back.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Minimum share of liquid waste that should be collected </t>
-  </si>
-  <si>
-    <t>LWTGEN</t>
-  </si>
-  <si>
-    <t>COLLWT</t>
-  </si>
-  <si>
-    <t>Variable Costs</t>
-  </si>
-  <si>
-    <t>Variable Cost of crops technologies</t>
-  </si>
-  <si>
-    <t>VariableCost</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LNDPLAHR ; LNDPLALR ; LNDMAIHR ; LNDMAILR ; LNDCASHR ; LNDCASLR ; LNDBEAHR ; LNDBEALR ; LNDCOFHR ; LNDCOFLR ; LNDGROHR ; LNDGROLR ; LNDPTSHR ; LNDPTSLR ; LNDSUNHR ; LNDSUNLR ; LNDOTCHR ; LNDOTCLR ; LNDSORHR ; LNDSORLR ; LNDSESHR ; LNDSESLR ; LNDRICHR ; LNDRICHI ; LNDRICLR; LNDSOYHR ; LNDSOYLR ; LNDVEGHR ; LNDVEGLR
-</t>
-  </si>
-  <si>
-    <t>Fixed Costs</t>
-  </si>
-  <si>
-    <t>Fixed Cost of crops technologies</t>
-  </si>
-  <si>
-    <t>FixedCost</t>
-  </si>
-  <si>
-    <t>LNDPLAHR ; LNDPLALR ; LNDMAIHR ; LNDMAILR ; LNDCASHR ; LNDCASLR ; LNDBEAHR ; LNDBEALR ; LNDCOFHR ; LNDCOFLR ; LNDGROHR ; LNDGROLR ; LNDPTSHR ; LNDPTSLR ; LNDSUNHR ; LNDSUNLR ; LNDOTCHR ; LNDOTCLR ; LNDSORHR ; LNDSORLR ; LNDSESHR ; LNDSESLR ; LNDRICHR ; LNDRICHI ; LNDRICLR; LNDSOYHR ; LNDSOYLR ; LNDVEGHR ; LNDVEGLR</t>
-  </si>
-  <si>
-    <t>Capital Costs</t>
-  </si>
-  <si>
-    <t>Capital Cost of electric vehicles technologies</t>
-  </si>
-  <si>
-    <t>CapitalCost</t>
-  </si>
-  <si>
-    <t>TRAELCCARCUR ; TRAELCCARNEW ; TRAELCMCYCUR ; TRAELCMCYNEW ; TRAELCMNBCUR ; TRAELCMNBNEW ; TRAELCBUSCUR ; TRAELCBUSNEW ; TRAELCLTRCUR ; TRAELCLTRNEW ; TRAELCMTRCUR ; TRAELCMTRNEW ; TRAELCHTRCUR ; TRAELCHTRNEW</t>
-  </si>
-  <si>
-    <t>Fixed Cost of electric vehicles technologies</t>
-  </si>
-  <si>
-    <t>Capital Cost of ICE vehicles technologies</t>
-  </si>
-  <si>
-    <t>TRADSLCARCUR ; TRALPGCARNEW ; TRADSLCARNEW ; TRADSLMCYNEW ; TRADSLMNBCUR ; TRALPGMNBNEW ; TRADSLMNBNEW ; TRADSHMNBNEW ; TRADSLBUSCUR ; TRADSLBUSNEW ; TRALPGBUSNEW ; TRADSLBUSNEW ; TRADSLLTRCUR ; TRADSLLTRNEW ; TRADSHLTRNEW ; TRADSLMTRCUR ; TRADSLMTRNEW ; TRADSLHTRCUR ; TRADSLHTRNEW</t>
-  </si>
-  <si>
-    <t>Fixed Cost of ICE vehicles technologies</t>
-  </si>
-  <si>
-    <t>Demand Growth</t>
-  </si>
-  <si>
-    <t>Changes in demand magnitude</t>
-  </si>
-  <si>
-    <t>AccumulatedAnnualDemand</t>
-  </si>
-  <si>
-    <t>RESLGTR ; RESLGTU ; RESCKNR ; RESCKNU ; RESSPHR ; RESWTHR ; RESWTHU ; RESCOLU ; RESELCOTHR ; RESELCOTHU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Import Cost of fuels </t>
-  </si>
-  <si>
-    <t>IMPDSL ; IMPGSL ; IMPKER ; IMPHFO ; IMPLPG</t>
-  </si>
-  <si>
-    <t>Input Activity Ratio</t>
-  </si>
-  <si>
-    <t>Activity ratio of inputs</t>
-  </si>
-  <si>
-    <t>InputActivityRatio</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> INDOTHPLT ; INDMTRPLT ;  INDCHMPLT ; INDFBTPLT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INDOTHHTH ; INDOTHMDR ; INDELC ; INDMTRHTH ; INDMTRMDR ; INDELC ; INDCHMHTH ; INDCHMMDR ; INDELC ; INDFBTHTH ; INDELC ; INDFBTMDR </t>
-  </si>
-  <si>
-    <t>Capital Cost of Steel direct electric arc furnance with hydrogen, Capital Cost of cement industry kilns with CCS</t>
-  </si>
-  <si>
-    <t>INDIRSHDGDRI ; INDNGSKLNCCS ; INDBIOKLNCCS ; INDCOAKLNCCS</t>
-  </si>
-  <si>
-    <t>Capital Cost of Steel direct electric arc furnance with natural gas technologies , Capital Cost of cement industry kilns without CCS</t>
-  </si>
-  <si>
-    <t>INDIRSNGSDRI ; INDWSTKLN ; INDHFOKLN ; INDNGSKLN ; INDBIOKLN ; INDKLNCOA</t>
-  </si>
-  <si>
-    <t>Output Activity Ratio</t>
-  </si>
-  <si>
-    <t>Activity ratio of outputs</t>
-  </si>
-  <si>
-    <t>OutputActivityRatio</t>
-  </si>
-  <si>
-    <t>CRPPLA ; CRPMAI ; CRPCAS ; CRPBEA ; CRPCOF ; CRPGRO ; CRPPTS ; CRPSUN ; CRPOTC ; CRPSOR ; CRPSES ; CRPRIC ; CRPSOY ; CRPVEG</t>
-  </si>
-  <si>
-    <t>parameter</t>
-  </si>
-  <si>
-    <t>YearSplit</t>
-  </si>
-  <si>
-    <t>DiscountRate</t>
-  </si>
-  <si>
-    <t>DiscountRateIdv</t>
-  </si>
-  <si>
-    <t>TradeRoute</t>
-  </si>
-  <si>
-    <t>DepreciationMethod</t>
-  </si>
-  <si>
-    <t>Conversionls</t>
-  </si>
-  <si>
-    <t>Conversionld</t>
-  </si>
-  <si>
-    <t>Conversionlh</t>
-  </si>
-  <si>
-    <t>DaySplit</t>
-  </si>
-  <si>
-    <t>DaysInDayType</t>
-  </si>
-  <si>
-    <t>SpecifiedAnnualDemand</t>
-  </si>
-  <si>
-    <t>SpecifiedDemandProfile</t>
-  </si>
-  <si>
-    <t>CapacityToActivityUnit</t>
-  </si>
-  <si>
-    <t>CapitalRecoveryFactor</t>
-  </si>
-  <si>
-    <t>CapacityOfOneTechnologyUnit</t>
-  </si>
-  <si>
-    <t>CapacityFactor</t>
-  </si>
-  <si>
-    <t>AvailabilityFactor</t>
-  </si>
-  <si>
-    <t>OperationalLife</t>
-  </si>
-  <si>
-    <t>ResidualCapacity</t>
-  </si>
-  <si>
-    <t>InputToNewCapacityRatio</t>
-  </si>
-  <si>
-    <t>InputToTotalCapacityRatio</t>
-  </si>
-  <si>
-    <t>PvAnnuity</t>
-  </si>
-  <si>
-    <t>CapitalCostStorage</t>
-  </si>
-  <si>
-    <t>TotalAnnualMaxCapacity</t>
-  </si>
-  <si>
-    <t>TotalAnnualMinCapacity</t>
-  </si>
-  <si>
-    <t>TotalAnnualMaxCapacityInvestment</t>
-  </si>
-  <si>
-    <t>TotalAnnualMinCapacityInvestment</t>
-  </si>
-  <si>
-    <t>TotalTechnologyAnnualActivityUpperLimit</t>
-  </si>
-  <si>
-    <t>TotalTechnologyAnnualActivityLowerLimit</t>
-  </si>
-  <si>
-    <t>TotalTechnologyModelPeriodActivityUpperLimit</t>
-  </si>
-  <si>
-    <t>TotalTechnologyModelPeriodActivityLowerLimit</t>
-  </si>
-  <si>
-    <t>EmissionActivityRatio</t>
-  </si>
-  <si>
-    <t>AnnualEmissionLimit</t>
-  </si>
-  <si>
-    <t>ModelPeriodEmissionLimit</t>
-  </si>
-  <si>
-    <t>EmissionsPenalty</t>
-  </si>
-  <si>
-    <t>EmissionToActivityChangeRatio</t>
-  </si>
-  <si>
-    <t>TechnologyFromStorage</t>
-  </si>
-  <si>
-    <t>TechnologyToStorage</t>
-  </si>
-  <si>
-    <t>StorageLevelStart</t>
-  </si>
-  <si>
-    <t>MinStorageCharge</t>
-  </si>
-  <si>
-    <t>OperationalLifeStorage</t>
-  </si>
-  <si>
-    <t>ResidualStorageCapacity</t>
-  </si>
-  <si>
-    <t>TechnologyActivityIncreaseByModeLimit</t>
-  </si>
-  <si>
-    <t>TechnologyActivityDecreaseByModeLimit</t>
-  </si>
-  <si>
-    <t>TechnologyActivityByModeLowerLimit</t>
-  </si>
-  <si>
-    <t>TechnologyActivityByModeUpperLimit</t>
-  </si>
-  <si>
-    <t>UDCConstant</t>
-  </si>
-  <si>
     <t>UDCMultiplierNewCapacity</t>
   </si>
   <si>
-    <t>UDCMultiplierTotalCapacity</t>
-  </si>
-  <si>
     <t>UDCTag</t>
   </si>
   <si>
@@ -672,15 +698,6 @@
   </si>
   <si>
     <t>TotalDiscountedStorageCost</t>
-  </si>
-  <si>
-    <t>cplex</t>
-  </si>
-  <si>
-    <t>Scenario1</t>
-  </si>
-  <si>
-    <t>model.v.5.3.txt</t>
   </si>
 </sst>
 </file>
@@ -1376,752 +1393,756 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:R130"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="35.4" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.5546875" style="3" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" style="3" customWidth="1"/>
+    <col min="1" max="1" width="9.5703125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" style="3" customWidth="1"/>
     <col min="3" max="3" width="44" style="20" customWidth="1"/>
-    <col min="4" max="4" width="34.88671875" style="3" customWidth="1"/>
-    <col min="5" max="5" width="27.44140625" style="3" customWidth="1"/>
-    <col min="6" max="7" width="32.109375" style="3" customWidth="1"/>
-    <col min="8" max="8" width="13.5546875" style="3" customWidth="1"/>
-    <col min="9" max="9" width="14.44140625" style="3" customWidth="1"/>
+    <col min="4" max="4" width="34.85546875" style="3" customWidth="1"/>
+    <col min="5" max="5" width="27.42578125" style="3" customWidth="1"/>
+    <col min="6" max="7" width="32.140625" style="3" customWidth="1"/>
+    <col min="8" max="8" width="13.5703125" style="3" customWidth="1"/>
+    <col min="9" max="9" width="14.42578125" style="3" customWidth="1"/>
     <col min="10" max="10" width="54" style="3" customWidth="1"/>
-    <col min="11" max="11" width="14.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="79.6640625" style="20" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="79.7109375" style="20" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="49" style="20" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="45.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="45.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="44" style="20" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="74.109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="31.6640625" style="3" customWidth="1"/>
-    <col min="18" max="18" width="13.33203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="19" max="21" width="8.88671875" style="3" customWidth="1"/>
-    <col min="22" max="16384" width="8.88671875" style="3"/>
+    <col min="16" max="16" width="74.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="31.7109375" style="3" customWidth="1"/>
+    <col min="18" max="18" width="13.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="19" max="20" width="8.85546875" style="3" customWidth="1"/>
+    <col min="21" max="16384" width="8.85546875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F1" s="16" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G1" s="16" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H1" s="16" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="I1" s="16" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="J1" s="16" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K1" s="18" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="L1" s="17" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="M1" s="17" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="N1" s="16" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="O1" s="17" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="P1" s="16" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="Q1" s="16" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="R1" s="16" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="2" spans="1:18" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="36">
         <v>1</v>
       </c>
       <c r="B2" s="25" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C2" s="26" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D2" s="25" t="s">
-        <v>190</v>
+        <v>40</v>
       </c>
       <c r="E2" s="25" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F2" s="25" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="G2" s="25">
-        <v>2026</v>
+        <v>2028</v>
       </c>
       <c r="H2" s="25">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="I2" s="25">
         <v>1</v>
       </c>
       <c r="J2" s="25" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="K2" s="27" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="L2" s="28" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="M2" s="26" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="N2" s="26" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O2" s="26" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="P2" s="25"/>
       <c r="Q2" s="25"/>
       <c r="R2" s="25"/>
     </row>
-    <row r="3" spans="1:18" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="36">
         <v>2</v>
       </c>
       <c r="B3" s="25" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C3" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="D3" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="E3" s="25" t="s">
+        <v>41</v>
+      </c>
+      <c r="F3" s="25" t="s">
+        <v>42</v>
+      </c>
+      <c r="G3" s="25">
+        <v>2028</v>
+      </c>
+      <c r="H3" s="25">
+        <v>0.5</v>
+      </c>
+      <c r="I3" s="25">
+        <v>1.2</v>
+      </c>
+      <c r="J3" s="25" t="s">
+        <v>43</v>
+      </c>
+      <c r="K3" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="L3" s="29" t="s">
+        <v>49</v>
+      </c>
+      <c r="M3" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="D3" s="25" t="s">
-        <v>190</v>
-      </c>
-      <c r="E3" s="25" t="s">
-        <v>38</v>
-      </c>
-      <c r="F3" s="25" t="s">
-        <v>39</v>
-      </c>
-      <c r="G3" s="25">
-        <v>2026</v>
-      </c>
-      <c r="H3" s="25">
-        <v>0.6</v>
-      </c>
-      <c r="I3" s="25">
-        <v>1</v>
-      </c>
-      <c r="J3" s="25" t="s">
-        <v>40</v>
-      </c>
-      <c r="K3" s="27" t="s">
-        <v>41</v>
-      </c>
-      <c r="L3" s="29" t="s">
+      <c r="N3" s="26" t="s">
+        <v>46</v>
+      </c>
+      <c r="O3" s="26" t="s">
         <v>47</v>
-      </c>
-      <c r="M3" s="26" t="s">
-        <v>48</v>
-      </c>
-      <c r="N3" s="26" t="s">
-        <v>44</v>
-      </c>
-      <c r="O3" s="26" t="s">
-        <v>45</v>
       </c>
       <c r="P3" s="25"/>
       <c r="Q3" s="25"/>
       <c r="R3" s="25"/>
     </row>
-    <row r="4" spans="1:18" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="36">
         <v>3</v>
       </c>
       <c r="B4" s="26" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C4" s="26" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D4" s="25" t="s">
-        <v>190</v>
+        <v>40</v>
       </c>
       <c r="E4" s="25" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F4" s="25" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="G4" s="25">
-        <v>2026</v>
+        <v>2028</v>
       </c>
       <c r="H4" s="25">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="I4" s="25">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="J4" s="30" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="K4" s="27" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="L4" s="31" t="s">
-        <v>52</v>
-      </c>
-      <c r="M4" s="29">
-        <v>1</v>
-      </c>
-      <c r="N4" s="26"/>
+        <v>53</v>
+      </c>
+      <c r="M4" s="29" t="s">
+        <v>46</v>
+      </c>
+      <c r="N4" s="26" t="s">
+        <v>46</v>
+      </c>
       <c r="O4" s="26" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="P4" s="25"/>
       <c r="Q4" s="25"/>
       <c r="R4" s="25"/>
     </row>
-    <row r="5" spans="1:18" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="36">
         <v>4</v>
       </c>
       <c r="B5" s="26" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C5" s="26" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D5" s="25" t="s">
-        <v>190</v>
+        <v>40</v>
       </c>
       <c r="E5" s="25" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F5" s="25" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="G5" s="25">
-        <v>2026</v>
+        <v>2028</v>
       </c>
       <c r="H5" s="25">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="I5" s="25">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="J5" s="30" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="K5" s="27" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="L5" s="31" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="M5" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="N5" s="26"/>
+        <v>58</v>
+      </c>
+      <c r="N5" s="26" t="s">
+        <v>46</v>
+      </c>
       <c r="O5" s="26" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="P5" s="25"/>
       <c r="Q5" s="25"/>
       <c r="R5" s="25"/>
     </row>
-    <row r="6" spans="1:18" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="36">
         <v>5</v>
       </c>
       <c r="B6" s="26" t="s">
-        <v>57</v>
+        <v>38</v>
       </c>
       <c r="C6" s="26" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D6" s="25" t="s">
-        <v>190</v>
+        <v>40</v>
       </c>
       <c r="E6" s="25" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F6" s="25" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="G6" s="25">
-        <v>2026</v>
+        <v>2028</v>
       </c>
       <c r="H6" s="30">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="I6" s="30">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="J6" s="30" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="K6" s="27" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="L6" s="29" t="s">
         <v>60</v>
       </c>
       <c r="M6" s="29" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N6" s="26" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O6" s="26" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="P6" s="25"/>
       <c r="Q6" s="25"/>
       <c r="R6" s="25"/>
     </row>
-    <row r="7" spans="1:18" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="36">
         <v>6</v>
       </c>
       <c r="B7" s="26" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C7" s="26" t="s">
         <v>61</v>
       </c>
       <c r="D7" s="25" t="s">
-        <v>190</v>
+        <v>40</v>
       </c>
       <c r="E7" s="25" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F7" s="25" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="G7" s="25">
-        <v>2026</v>
+        <v>2028</v>
       </c>
       <c r="H7" s="30">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="I7" s="30">
         <v>1.2</v>
       </c>
       <c r="J7" s="30" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="K7" s="27" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="L7" s="29" t="s">
         <v>60</v>
       </c>
       <c r="M7" s="29" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N7" s="26" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O7" s="26" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="P7" s="25"/>
       <c r="Q7" s="25"/>
       <c r="R7" s="25"/>
     </row>
-    <row r="8" spans="1:18" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="36">
         <v>7</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C8" s="26" t="s">
         <v>62</v>
       </c>
       <c r="D8" s="25" t="s">
-        <v>190</v>
+        <v>40</v>
       </c>
       <c r="E8" s="25" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F8" s="25" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="G8" s="25">
-        <v>2026</v>
+        <v>2028</v>
       </c>
       <c r="H8" s="30">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="I8" s="30">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="J8" s="30" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="K8" s="27" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="L8" s="29" t="s">
         <v>63</v>
       </c>
       <c r="M8" s="29" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="N8" s="26" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O8" s="26" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="P8" s="25"/>
       <c r="Q8" s="25"/>
       <c r="R8" s="25"/>
     </row>
-    <row r="9" spans="1:18" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="36">
         <v>8</v>
       </c>
       <c r="B9" s="32" t="s">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="C9" s="34" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D9" s="32" t="s">
-        <v>190</v>
+        <v>40</v>
       </c>
       <c r="E9" s="32" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F9" s="32" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="G9" s="32">
-        <v>2026</v>
+        <v>2030</v>
       </c>
       <c r="H9" s="32">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="I9" s="32">
         <v>1.1000000000000001</v>
       </c>
       <c r="J9" s="32" t="s">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="K9" s="33" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="L9" s="35" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="M9" s="34" t="s">
-        <v>44</v>
+        <v>68</v>
       </c>
       <c r="N9" s="34" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O9" s="34" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="P9" s="32"/>
       <c r="Q9" s="32"/>
       <c r="R9" s="32"/>
     </row>
-    <row r="10" spans="1:18" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="36">
         <v>9</v>
       </c>
       <c r="B10" s="32" t="s">
-        <v>65</v>
+        <v>38</v>
       </c>
       <c r="C10" s="34" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D10" s="32" t="s">
-        <v>190</v>
+        <v>40</v>
       </c>
       <c r="E10" s="32" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F10" s="32" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="G10" s="32">
-        <v>2026</v>
+        <v>2028</v>
       </c>
       <c r="H10" s="32">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="I10" s="32">
-        <v>1.2</v>
+        <v>3</v>
       </c>
       <c r="J10" s="32" t="s">
+        <v>43</v>
+      </c>
+      <c r="K10" s="33" t="s">
+        <v>44</v>
+      </c>
+      <c r="L10" s="35" t="s">
         <v>67</v>
       </c>
-      <c r="K10" s="33" t="s">
-        <v>41</v>
-      </c>
-      <c r="L10" s="35" t="s">
-        <v>68</v>
-      </c>
       <c r="M10" s="34" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N10" s="34" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O10" s="34" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="P10" s="32"/>
       <c r="Q10" s="32"/>
       <c r="R10" s="32"/>
     </row>
-    <row r="11" spans="1:18" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="36">
         <v>10</v>
       </c>
       <c r="B11" s="32" t="s">
-        <v>49</v>
+        <v>70</v>
       </c>
       <c r="C11" s="34" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D11" s="32" t="s">
-        <v>190</v>
+        <v>40</v>
       </c>
       <c r="E11" s="32" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F11" s="32" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="G11" s="32">
-        <v>2026</v>
+        <v>2028</v>
       </c>
       <c r="H11" s="32">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="I11" s="32">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="J11" s="32" t="s">
-        <v>51</v>
+        <v>72</v>
       </c>
       <c r="K11" s="33" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="L11" s="35" t="s">
-        <v>70</v>
-      </c>
-      <c r="M11" s="32">
-        <v>1</v>
+        <v>73</v>
+      </c>
+      <c r="M11" s="32" t="s">
+        <v>74</v>
       </c>
       <c r="N11" s="34" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O11" s="34" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="P11" s="32"/>
       <c r="Q11" s="32"/>
       <c r="R11" s="32"/>
     </row>
-    <row r="12" spans="1:18" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="36">
         <v>11</v>
       </c>
       <c r="B12" s="32" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C12" s="34" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D12" s="32" t="s">
-        <v>190</v>
+        <v>40</v>
       </c>
       <c r="E12" s="32" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F12" s="32" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="G12" s="32">
-        <v>2026</v>
+        <v>2028</v>
       </c>
       <c r="H12" s="32">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="I12" s="32">
         <v>1.2</v>
       </c>
       <c r="J12" s="32" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="K12" s="33" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="L12" s="35" t="s">
-        <v>74</v>
+        <v>60</v>
       </c>
       <c r="M12" s="34" t="s">
-        <v>75</v>
-      </c>
-      <c r="N12" s="34">
-        <v>1</v>
+        <v>78</v>
+      </c>
+      <c r="N12" s="34" t="s">
+        <v>58</v>
       </c>
       <c r="O12" s="34" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="P12" s="32"/>
       <c r="Q12" s="32"/>
       <c r="R12" s="32"/>
     </row>
-    <row r="13" spans="1:18" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="36">
         <v>12</v>
       </c>
       <c r="B13" s="32" t="s">
-        <v>57</v>
+        <v>79</v>
       </c>
       <c r="C13" s="34" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D13" s="32" t="s">
-        <v>190</v>
+        <v>40</v>
       </c>
       <c r="E13" s="32" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F13" s="32" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="G13" s="32">
-        <v>2026</v>
+        <v>2028</v>
       </c>
       <c r="H13" s="32">
         <v>0.8</v>
       </c>
       <c r="I13" s="32">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="J13" s="32" t="s">
-        <v>59</v>
+        <v>81</v>
       </c>
       <c r="K13" s="33" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="L13" s="35" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="M13" s="34" t="s">
-        <v>44</v>
+        <v>83</v>
       </c>
       <c r="N13" s="34" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="O13" s="34" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="P13" s="32"/>
       <c r="Q13" s="32"/>
       <c r="R13" s="32"/>
     </row>
-    <row r="14" spans="1:18" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:18" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="36">
         <v>13</v>
       </c>
       <c r="B14" s="32" t="s">
-        <v>57</v>
+        <v>84</v>
       </c>
       <c r="C14" s="32" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D14" s="32" t="s">
-        <v>190</v>
+        <v>40</v>
       </c>
       <c r="E14" s="32" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F14" s="32" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="G14" s="32">
-        <v>2026</v>
+        <v>2028</v>
       </c>
       <c r="H14" s="32">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="I14" s="32">
-        <v>1.3</v>
+        <v>8</v>
       </c>
       <c r="J14" s="32" t="s">
-        <v>59</v>
+        <v>85</v>
       </c>
       <c r="K14" s="33" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="L14" s="34" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="M14" s="34" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N14" s="32" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O14" s="34" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="P14" s="32"/>
       <c r="Q14" s="32"/>
       <c r="R14" s="32"/>
     </row>
-    <row r="15" spans="1:18" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:18" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="36">
         <v>14</v>
       </c>
       <c r="B15" s="32" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="C15" s="32" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="D15" s="32" t="s">
-        <v>190</v>
+        <v>40</v>
       </c>
       <c r="E15" s="32" t="s">
-        <v>38</v>
+        <v>88</v>
       </c>
       <c r="F15" s="32" t="s">
-        <v>39</v>
+        <v>89</v>
       </c>
       <c r="G15" s="32">
-        <v>2026</v>
+        <v>2036</v>
       </c>
       <c r="H15" s="32">
         <v>0.8</v>
@@ -2130,69 +2151,99 @@
         <v>1.2</v>
       </c>
       <c r="J15" s="32" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="K15" s="33" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="L15" s="34" t="s">
-        <v>52</v>
+        <v>91</v>
       </c>
       <c r="M15" s="34" t="s">
-        <v>83</v>
-      </c>
-      <c r="N15" s="34">
-        <v>1</v>
+        <v>74</v>
+      </c>
+      <c r="N15" s="34" t="s">
+        <v>46</v>
       </c>
       <c r="O15" s="34" t="s">
-        <v>45</v>
+        <v>92</v>
       </c>
       <c r="P15" s="32"/>
       <c r="Q15" s="32"/>
       <c r="R15" s="32"/>
     </row>
-    <row r="16" spans="1:18" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="36"/>
-      <c r="B16" s="32"/>
-      <c r="C16" s="32"/>
-      <c r="D16" s="32"/>
-      <c r="E16" s="32"/>
-      <c r="F16" s="32"/>
-      <c r="G16" s="32"/>
-      <c r="H16" s="32"/>
-      <c r="I16" s="32"/>
-      <c r="J16" s="32"/>
-      <c r="K16" s="33"/>
-      <c r="L16" s="34"/>
-      <c r="M16" s="34"/>
-      <c r="N16" s="34"/>
-      <c r="O16" s="34"/>
+    <row r="16" spans="1:18" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="36">
+        <v>15</v>
+      </c>
+      <c r="B16" s="32" t="s">
+        <v>93</v>
+      </c>
+      <c r="C16" s="32" t="s">
+        <v>94</v>
+      </c>
+      <c r="D16" s="32" t="s">
+        <v>40</v>
+      </c>
+      <c r="E16" s="32" t="s">
+        <v>41</v>
+      </c>
+      <c r="F16" s="32" t="s">
+        <v>42</v>
+      </c>
+      <c r="G16" s="32">
+        <v>2028</v>
+      </c>
+      <c r="H16" s="32">
+        <v>0.8</v>
+      </c>
+      <c r="I16" s="32">
+        <v>1.2</v>
+      </c>
+      <c r="J16" s="32" t="s">
+        <v>95</v>
+      </c>
+      <c r="K16" s="33" t="s">
+        <v>44</v>
+      </c>
+      <c r="L16" s="34" t="s">
+        <v>91</v>
+      </c>
+      <c r="M16" s="34" t="s">
+        <v>46</v>
+      </c>
+      <c r="N16" s="34" t="s">
+        <v>46</v>
+      </c>
+      <c r="O16" s="34" t="s">
+        <v>47</v>
+      </c>
       <c r="P16" s="38"/>
       <c r="Q16" s="38"/>
       <c r="R16" s="37"/>
     </row>
-    <row r="17" spans="2:17" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:17" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C17" s="3"/>
       <c r="K17" s="21"/>
       <c r="N17" s="20"/>
       <c r="P17" s="20"/>
       <c r="Q17" s="20"/>
     </row>
-    <row r="18" spans="2:17" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:17" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C18" s="3"/>
       <c r="K18" s="21"/>
       <c r="N18" s="20"/>
       <c r="P18" s="20"/>
       <c r="Q18" s="20"/>
     </row>
-    <row r="19" spans="2:17" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:17" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C19" s="3"/>
       <c r="K19" s="21"/>
       <c r="N19" s="20"/>
       <c r="P19" s="20"/>
       <c r="Q19" s="20"/>
     </row>
-    <row r="20" spans="2:17" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:17" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="39"/>
       <c r="C20" s="39"/>
       <c r="D20" s="39"/>
@@ -2208,7 +2259,7 @@
       <c r="N20" s="41"/>
       <c r="O20" s="41"/>
     </row>
-    <row r="21" spans="2:17" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:17" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="39"/>
       <c r="C21" s="39"/>
       <c r="D21" s="39"/>
@@ -2224,7 +2275,7 @@
       <c r="N21" s="41"/>
       <c r="O21" s="41"/>
     </row>
-    <row r="22" spans="2:17" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:17" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="39"/>
       <c r="C22" s="39"/>
       <c r="D22" s="39"/>
@@ -2240,7 +2291,7 @@
       <c r="N22" s="41"/>
       <c r="O22" s="41"/>
     </row>
-    <row r="23" spans="2:17" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:17" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="39"/>
       <c r="C23" s="41"/>
       <c r="D23" s="39"/>
@@ -2256,7 +2307,7 @@
       <c r="N23" s="41"/>
       <c r="O23" s="41"/>
     </row>
-    <row r="24" spans="2:17" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:17" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="39"/>
       <c r="C24" s="41"/>
       <c r="D24" s="39"/>
@@ -2272,7 +2323,7 @@
       <c r="N24" s="41"/>
       <c r="O24" s="41"/>
     </row>
-    <row r="25" spans="2:17" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:17" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="39"/>
       <c r="C25" s="39"/>
       <c r="D25" s="39"/>
@@ -2288,7 +2339,7 @@
       <c r="N25" s="41"/>
       <c r="O25" s="41"/>
     </row>
-    <row r="26" spans="2:17" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:17" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="39"/>
       <c r="C26" s="41"/>
       <c r="D26" s="39"/>
@@ -2304,7 +2355,7 @@
       <c r="N26" s="41"/>
       <c r="O26" s="41"/>
     </row>
-    <row r="27" spans="2:17" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:17" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="39"/>
       <c r="C27" s="39"/>
       <c r="D27" s="39"/>
@@ -2320,7 +2371,7 @@
       <c r="N27" s="41"/>
       <c r="O27" s="41"/>
     </row>
-    <row r="28" spans="2:17" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:17" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="39"/>
       <c r="C28" s="41"/>
       <c r="D28" s="39"/>
@@ -2336,7 +2387,7 @@
       <c r="N28" s="41"/>
       <c r="O28" s="41"/>
     </row>
-    <row r="29" spans="2:17" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:17" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="39"/>
       <c r="C29" s="41"/>
       <c r="D29" s="39"/>
@@ -2352,7 +2403,7 @@
       <c r="N29" s="41"/>
       <c r="O29" s="41"/>
     </row>
-    <row r="30" spans="2:17" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:17" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="39"/>
       <c r="C30" s="39"/>
       <c r="D30" s="39"/>
@@ -2368,7 +2419,7 @@
       <c r="N30" s="41"/>
       <c r="O30" s="41"/>
     </row>
-    <row r="31" spans="2:17" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:17" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="39"/>
       <c r="C31" s="41"/>
       <c r="D31" s="39"/>
@@ -2384,7 +2435,7 @@
       <c r="N31" s="41"/>
       <c r="O31" s="41"/>
     </row>
-    <row r="32" spans="2:17" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:17" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="39"/>
       <c r="C32" s="41"/>
       <c r="D32" s="39"/>
@@ -2400,7 +2451,7 @@
       <c r="N32" s="41"/>
       <c r="O32" s="41"/>
     </row>
-    <row r="33" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="39"/>
       <c r="C33" s="39"/>
       <c r="D33" s="39"/>
@@ -2416,7 +2467,7 @@
       <c r="N33" s="41"/>
       <c r="O33" s="41"/>
     </row>
-    <row r="34" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" s="39"/>
       <c r="C34" s="41"/>
       <c r="D34" s="39"/>
@@ -2432,7 +2483,7 @@
       <c r="N34" s="41"/>
       <c r="O34" s="41"/>
     </row>
-    <row r="35" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="39"/>
       <c r="C35" s="41"/>
       <c r="D35" s="39"/>
@@ -2448,7 +2499,7 @@
       <c r="N35" s="41"/>
       <c r="O35" s="41"/>
     </row>
-    <row r="36" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="39"/>
       <c r="C36" s="41"/>
       <c r="D36" s="39"/>
@@ -2464,7 +2515,7 @@
       <c r="N36" s="41"/>
       <c r="O36" s="41"/>
     </row>
-    <row r="37" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="39"/>
       <c r="C37" s="41"/>
       <c r="D37" s="39"/>
@@ -2480,7 +2531,7 @@
       <c r="N37" s="41"/>
       <c r="O37" s="41"/>
     </row>
-    <row r="38" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="39"/>
       <c r="C38" s="39"/>
       <c r="D38" s="39"/>
@@ -2496,7 +2547,7 @@
       <c r="N38" s="41"/>
       <c r="O38" s="41"/>
     </row>
-    <row r="39" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="39"/>
       <c r="D39" s="39"/>
       <c r="E39" s="39"/>
@@ -2511,12 +2562,12 @@
       <c r="N39" s="41"/>
       <c r="O39" s="41"/>
     </row>
-    <row r="40" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F40" s="39"/>
       <c r="K40" s="23"/>
       <c r="N40" s="20"/>
     </row>
-    <row r="41" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B41" s="39"/>
       <c r="C41" s="41"/>
       <c r="D41" s="39"/>
@@ -2532,7 +2583,7 @@
       <c r="N41" s="41"/>
       <c r="O41" s="41"/>
     </row>
-    <row r="42" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B42" s="39"/>
       <c r="C42" s="41"/>
       <c r="D42" s="39"/>
@@ -2548,7 +2599,7 @@
       <c r="N42" s="41"/>
       <c r="O42" s="41"/>
     </row>
-    <row r="43" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B43" s="39"/>
       <c r="C43" s="41"/>
       <c r="D43" s="39"/>
@@ -2564,7 +2615,7 @@
       <c r="N43" s="41"/>
       <c r="O43" s="41"/>
     </row>
-    <row r="44" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B44" s="39"/>
       <c r="C44" s="41"/>
       <c r="D44" s="39"/>
@@ -2580,7 +2631,7 @@
       <c r="N44" s="41"/>
       <c r="O44" s="41"/>
     </row>
-    <row r="45" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="39"/>
       <c r="C45" s="39"/>
       <c r="D45" s="39"/>
@@ -2596,7 +2647,7 @@
       <c r="N45" s="41"/>
       <c r="O45" s="41"/>
     </row>
-    <row r="46" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B46" s="39"/>
       <c r="C46" s="41"/>
       <c r="D46" s="39"/>
@@ -2612,7 +2663,7 @@
       <c r="N46" s="41"/>
       <c r="O46" s="41"/>
     </row>
-    <row r="47" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B47" s="39"/>
       <c r="C47" s="41"/>
       <c r="D47" s="39"/>
@@ -2628,7 +2679,7 @@
       <c r="N47" s="41"/>
       <c r="O47" s="41"/>
     </row>
-    <row r="48" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B48" s="39"/>
       <c r="C48" s="39"/>
       <c r="D48" s="39"/>
@@ -2644,7 +2695,7 @@
       <c r="N48" s="41"/>
       <c r="O48" s="41"/>
     </row>
-    <row r="49" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F49" s="39"/>
       <c r="H49" s="39"/>
       <c r="I49" s="39"/>
@@ -2652,13 +2703,13 @@
       <c r="L49" s="22"/>
       <c r="N49" s="20"/>
     </row>
-    <row r="50" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F50" s="39"/>
       <c r="K50" s="21"/>
       <c r="L50" s="22"/>
       <c r="N50" s="20"/>
     </row>
-    <row r="51" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B51" s="39"/>
       <c r="C51" s="39"/>
       <c r="D51" s="39"/>
@@ -2674,223 +2725,225 @@
       <c r="N51" s="41"/>
       <c r="O51" s="41"/>
     </row>
-    <row r="52" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D52" s="20"/>
       <c r="F52" s="39"/>
       <c r="K52" s="21"/>
       <c r="L52" s="22"/>
       <c r="N52" s="20"/>
-    </row>
-    <row r="53" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="O52"/>
+    </row>
+    <row r="53" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D53" s="20"/>
       <c r="F53" s="39"/>
       <c r="K53" s="21"/>
       <c r="L53" s="22"/>
       <c r="N53" s="20"/>
-    </row>
-    <row r="54" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="O53"/>
+    </row>
+    <row r="54" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F54" s="39"/>
       <c r="K54" s="21"/>
       <c r="L54" s="22"/>
       <c r="N54" s="20"/>
     </row>
-    <row r="55" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F55" s="39"/>
       <c r="K55" s="21"/>
       <c r="L55" s="22"/>
       <c r="N55" s="20"/>
     </row>
-    <row r="56" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K56" s="21"/>
       <c r="L56" s="22"/>
       <c r="N56" s="20"/>
     </row>
-    <row r="57" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K57" s="21"/>
       <c r="L57" s="22"/>
       <c r="N57" s="20"/>
     </row>
-    <row r="58" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K58" s="21"/>
       <c r="L58" s="22"/>
       <c r="N58" s="20"/>
     </row>
-    <row r="59" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K59" s="21"/>
       <c r="L59" s="22"/>
       <c r="N59" s="20"/>
     </row>
-    <row r="60" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K60" s="21"/>
       <c r="L60" s="22"/>
       <c r="N60" s="20"/>
     </row>
-    <row r="61" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K61" s="21"/>
       <c r="L61" s="22"/>
       <c r="N61" s="20"/>
     </row>
-    <row r="62" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K62" s="21"/>
       <c r="L62" s="22"/>
       <c r="N62" s="20"/>
     </row>
-    <row r="63" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K63" s="21"/>
       <c r="L63" s="22"/>
       <c r="N63" s="20"/>
     </row>
-    <row r="64" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K64" s="21"/>
       <c r="L64" s="22"/>
       <c r="N64" s="20"/>
     </row>
-    <row r="65" spans="11:14" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="11:14" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K65" s="21"/>
       <c r="L65" s="22"/>
       <c r="N65" s="20"/>
     </row>
-    <row r="66" spans="11:14" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="11:14" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K66" s="21"/>
       <c r="L66" s="22"/>
       <c r="N66" s="20"/>
     </row>
-    <row r="67" spans="11:14" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="11:14" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K67" s="21"/>
       <c r="L67" s="22"/>
       <c r="N67" s="20"/>
     </row>
-    <row r="68" spans="11:14" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="11:14" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K68" s="21"/>
       <c r="L68" s="22"/>
       <c r="N68" s="20"/>
     </row>
-    <row r="69" spans="11:14" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="11:14" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K69" s="21"/>
       <c r="L69" s="22"/>
       <c r="N69" s="20"/>
     </row>
-    <row r="70" spans="11:14" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="11:14" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K70" s="21"/>
       <c r="L70" s="22"/>
       <c r="N70" s="20"/>
     </row>
-    <row r="71" spans="11:14" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="11:14" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K71" s="21"/>
       <c r="L71" s="22"/>
       <c r="N71" s="20"/>
     </row>
-    <row r="72" spans="11:14" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="11:14" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K72" s="21"/>
       <c r="L72" s="22"/>
       <c r="N72" s="20"/>
     </row>
-    <row r="73" spans="11:14" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="11:14" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K73" s="21"/>
       <c r="L73" s="22"/>
       <c r="N73" s="20"/>
     </row>
-    <row r="74" spans="11:14" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="11:14" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K74" s="21"/>
       <c r="L74" s="22"/>
       <c r="N74" s="20"/>
     </row>
-    <row r="75" spans="11:14" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="11:14" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K75" s="21"/>
       <c r="L75" s="22"/>
       <c r="N75" s="20"/>
     </row>
-    <row r="76" spans="11:14" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="11:14" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K76" s="21"/>
       <c r="L76" s="22"/>
       <c r="N76" s="20"/>
     </row>
-    <row r="77" spans="11:14" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="11:14" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K77" s="21"/>
       <c r="L77" s="22"/>
       <c r="N77" s="20"/>
     </row>
-    <row r="78" spans="11:14" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="11:14" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K78" s="21"/>
       <c r="L78" s="22"/>
       <c r="N78" s="20"/>
     </row>
-    <row r="79" spans="11:14" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="11:14" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K79" s="21"/>
       <c r="L79" s="22"/>
       <c r="N79" s="20"/>
     </row>
-    <row r="80" spans="11:14" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="11:14" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K80" s="21"/>
       <c r="L80" s="22"/>
       <c r="N80" s="20"/>
     </row>
-    <row r="81" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K81" s="21"/>
       <c r="L81" s="22"/>
       <c r="N81" s="20"/>
     </row>
-    <row r="82" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K82" s="21"/>
       <c r="L82" s="22"/>
       <c r="N82" s="20"/>
     </row>
-    <row r="83" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K83" s="21"/>
       <c r="L83" s="22"/>
       <c r="N83" s="20"/>
     </row>
-    <row r="84" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K84" s="21"/>
       <c r="L84" s="22"/>
       <c r="N84" s="20"/>
     </row>
-    <row r="85" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K85" s="21"/>
       <c r="L85" s="22"/>
       <c r="N85" s="20"/>
     </row>
-    <row r="86" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K86" s="21"/>
       <c r="L86" s="22"/>
       <c r="N86" s="20"/>
     </row>
-    <row r="87" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K87" s="21"/>
       <c r="L87" s="22"/>
       <c r="N87" s="20"/>
     </row>
-    <row r="88" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K88" s="21"/>
       <c r="L88" s="22"/>
       <c r="N88" s="20"/>
     </row>
-    <row r="89" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K89" s="21"/>
       <c r="L89" s="22"/>
       <c r="N89" s="20"/>
     </row>
-    <row r="90" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K90" s="21"/>
       <c r="L90" s="22"/>
       <c r="N90" s="20"/>
     </row>
-    <row r="91" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K91" s="21"/>
       <c r="L91" s="22"/>
       <c r="N91" s="20"/>
     </row>
-    <row r="92" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K92" s="21"/>
       <c r="L92" s="22"/>
       <c r="N92" s="20"/>
     </row>
-    <row r="93" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K93" s="21"/>
       <c r="L93" s="22"/>
       <c r="N93" s="20"/>
     </row>
-    <row r="94" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B94" s="19"/>
       <c r="E94" s="19"/>
       <c r="F94" s="19"/>
@@ -2904,7 +2957,7 @@
       <c r="N94" s="22"/>
       <c r="O94" s="22"/>
     </row>
-    <row r="95" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B95" s="19"/>
       <c r="E95" s="19"/>
       <c r="F95" s="19"/>
@@ -2918,7 +2971,7 @@
       <c r="N95" s="22"/>
       <c r="O95" s="22"/>
     </row>
-    <row r="96" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B96" s="19"/>
       <c r="E96" s="19"/>
       <c r="F96" s="19"/>
@@ -2932,7 +2985,7 @@
       <c r="N96" s="22"/>
       <c r="O96" s="22"/>
     </row>
-    <row r="97" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B97" s="19"/>
       <c r="E97" s="19"/>
       <c r="F97" s="19"/>
@@ -2946,7 +2999,7 @@
       <c r="N97" s="22"/>
       <c r="O97" s="22"/>
     </row>
-    <row r="98" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B98" s="19"/>
       <c r="E98" s="19"/>
       <c r="F98" s="19"/>
@@ -2960,7 +3013,7 @@
       <c r="N98" s="22"/>
       <c r="O98" s="22"/>
     </row>
-    <row r="99" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B99" s="19"/>
       <c r="E99" s="19"/>
       <c r="F99" s="19"/>
@@ -2974,7 +3027,7 @@
       <c r="N99" s="22"/>
       <c r="O99" s="22"/>
     </row>
-    <row r="100" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B100" s="19"/>
       <c r="E100" s="19"/>
       <c r="F100" s="19"/>
@@ -2988,7 +3041,7 @@
       <c r="N100" s="22"/>
       <c r="O100" s="22"/>
     </row>
-    <row r="101" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B101" s="19"/>
       <c r="E101" s="19"/>
       <c r="F101" s="19"/>
@@ -3002,7 +3055,7 @@
       <c r="N101" s="22"/>
       <c r="O101" s="22"/>
     </row>
-    <row r="102" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B102" s="19"/>
       <c r="E102" s="19"/>
       <c r="F102" s="19"/>
@@ -3016,7 +3069,7 @@
       <c r="N102" s="22"/>
       <c r="O102" s="22"/>
     </row>
-    <row r="103" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B103" s="19"/>
       <c r="E103" s="19"/>
       <c r="F103" s="19"/>
@@ -3030,7 +3083,7 @@
       <c r="N103" s="22"/>
       <c r="O103" s="22"/>
     </row>
-    <row r="104" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B104" s="19"/>
       <c r="E104" s="19"/>
       <c r="F104" s="19"/>
@@ -3044,7 +3097,7 @@
       <c r="N104" s="22"/>
       <c r="O104" s="22"/>
     </row>
-    <row r="105" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B105" s="19"/>
       <c r="E105" s="19"/>
       <c r="F105" s="19"/>
@@ -3058,7 +3111,7 @@
       <c r="N105" s="22"/>
       <c r="O105" s="22"/>
     </row>
-    <row r="106" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B106" s="19"/>
       <c r="E106" s="19"/>
       <c r="F106" s="19"/>
@@ -3072,7 +3125,7 @@
       <c r="N106" s="22"/>
       <c r="O106" s="22"/>
     </row>
-    <row r="107" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B107" s="19"/>
       <c r="E107" s="19"/>
       <c r="F107" s="19"/>
@@ -3086,7 +3139,7 @@
       <c r="N107" s="22"/>
       <c r="O107" s="22"/>
     </row>
-    <row r="108" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B108" s="19"/>
       <c r="E108" s="19"/>
       <c r="F108" s="19"/>
@@ -3100,7 +3153,7 @@
       <c r="N108" s="22"/>
       <c r="O108" s="22"/>
     </row>
-    <row r="109" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B109" s="19"/>
       <c r="E109" s="19"/>
       <c r="F109" s="19"/>
@@ -3114,26 +3167,26 @@
       <c r="N109" s="22"/>
       <c r="O109" s="22"/>
     </row>
-    <row r="110" spans="2:15" s="19" customFormat="1" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="2:15" s="19" customFormat="1" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K110" s="21"/>
       <c r="L110" s="22"/>
       <c r="M110" s="22"/>
       <c r="N110" s="22"/>
       <c r="O110" s="22"/>
     </row>
-    <row r="111" spans="2:15" s="19" customFormat="1" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="2:15" s="19" customFormat="1" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K111" s="21"/>
       <c r="L111" s="22"/>
       <c r="M111" s="22"/>
       <c r="N111" s="22"/>
       <c r="O111" s="22"/>
     </row>
-    <row r="112" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K112" s="23"/>
       <c r="L112" s="24"/>
       <c r="N112" s="20"/>
     </row>
-    <row r="113" spans="1:15" s="19" customFormat="1" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:15" s="19" customFormat="1" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="3"/>
       <c r="C113" s="20"/>
       <c r="D113" s="3"/>
@@ -3143,14 +3196,14 @@
       <c r="N113" s="22"/>
       <c r="O113" s="22"/>
     </row>
-    <row r="114" spans="1:15" s="19" customFormat="1" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:15" s="19" customFormat="1" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K114" s="21"/>
       <c r="L114" s="22"/>
       <c r="M114" s="22"/>
       <c r="N114" s="22"/>
       <c r="O114" s="22"/>
     </row>
-    <row r="115" spans="1:15" s="19" customFormat="1" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:15" s="19" customFormat="1" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="3"/>
       <c r="B115" s="3"/>
       <c r="C115" s="20"/>
@@ -3167,14 +3220,14 @@
       <c r="N115" s="20"/>
       <c r="O115" s="20"/>
     </row>
-    <row r="116" spans="1:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K116" s="21"/>
       <c r="L116" s="22"/>
       <c r="M116" s="22"/>
       <c r="N116" s="22"/>
       <c r="O116" s="22"/>
     </row>
-    <row r="117" spans="1:15" s="19" customFormat="1" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:15" s="19" customFormat="1" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="3"/>
       <c r="C117" s="20"/>
       <c r="D117" s="3"/>
@@ -3184,14 +3237,14 @@
       <c r="N117" s="22"/>
       <c r="O117" s="22"/>
     </row>
-    <row r="118" spans="1:15" s="19" customFormat="1" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:15" s="19" customFormat="1" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K118" s="21"/>
       <c r="L118" s="22"/>
       <c r="M118" s="22"/>
       <c r="N118" s="22"/>
       <c r="O118" s="22"/>
     </row>
-    <row r="119" spans="1:15" s="19" customFormat="1" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:15" s="19" customFormat="1" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="3"/>
       <c r="B119" s="3"/>
       <c r="C119" s="20"/>
@@ -3208,14 +3261,14 @@
       <c r="N119" s="20"/>
       <c r="O119" s="20"/>
     </row>
-    <row r="120" spans="1:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K120" s="21"/>
       <c r="L120" s="22"/>
       <c r="M120" s="22"/>
       <c r="N120" s="22"/>
       <c r="O120" s="22"/>
     </row>
-    <row r="121" spans="1:15" s="19" customFormat="1" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:15" s="19" customFormat="1" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="3"/>
       <c r="C121" s="20"/>
       <c r="D121" s="3"/>
@@ -3225,14 +3278,14 @@
       <c r="N121" s="22"/>
       <c r="O121" s="22"/>
     </row>
-    <row r="122" spans="1:15" s="19" customFormat="1" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:15" s="19" customFormat="1" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K122" s="21"/>
       <c r="L122" s="22"/>
       <c r="M122" s="22"/>
       <c r="N122" s="22"/>
       <c r="O122" s="22"/>
     </row>
-    <row r="123" spans="1:15" s="19" customFormat="1" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:15" s="19" customFormat="1" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123" s="3"/>
       <c r="B123" s="3"/>
       <c r="C123" s="20"/>
@@ -3249,14 +3302,14 @@
       <c r="N123" s="20"/>
       <c r="O123" s="20"/>
     </row>
-    <row r="124" spans="1:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K124" s="21"/>
       <c r="L124" s="22"/>
       <c r="M124" s="22"/>
       <c r="N124" s="22"/>
       <c r="O124" s="22"/>
     </row>
-    <row r="125" spans="1:15" s="19" customFormat="1" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:15" s="19" customFormat="1" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="3"/>
       <c r="C125" s="20"/>
       <c r="D125" s="3"/>
@@ -3266,14 +3319,14 @@
       <c r="N125" s="22"/>
       <c r="O125" s="22"/>
     </row>
-    <row r="126" spans="1:15" s="19" customFormat="1" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:15" s="19" customFormat="1" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K126" s="21"/>
       <c r="L126" s="22"/>
       <c r="M126" s="22"/>
       <c r="N126" s="22"/>
       <c r="O126" s="22"/>
     </row>
-    <row r="127" spans="1:15" s="19" customFormat="1" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:15" s="19" customFormat="1" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127" s="3"/>
       <c r="B127" s="3"/>
       <c r="C127" s="20"/>
@@ -3290,21 +3343,21 @@
       <c r="N127" s="20"/>
       <c r="O127" s="20"/>
     </row>
-    <row r="128" spans="1:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K128" s="21"/>
       <c r="L128" s="22"/>
       <c r="M128" s="22"/>
       <c r="N128" s="22"/>
       <c r="O128" s="22"/>
     </row>
-    <row r="129" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K129" s="21"/>
       <c r="L129" s="22"/>
       <c r="M129" s="22"/>
       <c r="N129" s="22"/>
       <c r="O129" s="22"/>
     </row>
-    <row r="130" spans="2:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="2:15" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B130" s="19"/>
       <c r="E130" s="19"/>
       <c r="F130" s="19"/>
@@ -3329,20 +3382,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:O2"/>
-  <sheetFormatPr defaultColWidth="15.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="15.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="24.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="24.28515625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="18" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3389,9 +3442,9 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="72.599999999999994" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15" ht="72.599999999999994" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>15</v>
@@ -3400,10 +3453,10 @@
         <v>1</v>
       </c>
       <c r="D2" s="8">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E2" s="9">
-        <v>8</v>
+        <v>54</v>
       </c>
       <c r="F2" s="12" t="s">
         <v>16</v>
@@ -3412,19 +3465,19 @@
         <v>16</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>189</v>
+        <v>17</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>191</v>
+        <v>18</v>
       </c>
       <c r="J2" s="13" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="K2" s="13"/>
       <c r="L2" s="13"/>
       <c r="M2" s="15"/>
       <c r="N2" s="13">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O2" s="15">
         <v>3000</v>
@@ -3438,190 +3491,190 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:BG5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:59" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="B1" t="s">
-        <v>85</v>
+        <v>97</v>
       </c>
       <c r="C1" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="D1" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="E1" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="F1" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="G1" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="H1" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="I1" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="J1" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="K1" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="L1" t="s">
         <v>95</v>
       </c>
       <c r="M1" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="N1" t="s">
-        <v>67</v>
+        <v>107</v>
       </c>
       <c r="O1" t="s">
-        <v>97</v>
+        <v>108</v>
       </c>
       <c r="P1" t="s">
-        <v>98</v>
+        <v>109</v>
       </c>
       <c r="Q1" t="s">
-        <v>99</v>
+        <v>110</v>
       </c>
       <c r="R1" t="s">
-        <v>100</v>
+        <v>72</v>
       </c>
       <c r="S1" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="T1" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="U1" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="V1" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="W1" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="X1" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="Y1" t="s">
-        <v>82</v>
+        <v>116</v>
       </c>
       <c r="Z1" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="AA1" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="AB1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="AC1" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="AD1" t="s">
-        <v>107</v>
+        <v>118</v>
       </c>
       <c r="AE1" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
       <c r="AF1" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
       <c r="AG1" t="s">
-        <v>110</v>
+        <v>121</v>
       </c>
       <c r="AH1" t="s">
-        <v>111</v>
+        <v>122</v>
       </c>
       <c r="AI1" t="s">
-        <v>112</v>
+        <v>123</v>
       </c>
       <c r="AJ1" t="s">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="AK1" t="s">
-        <v>114</v>
+        <v>125</v>
       </c>
       <c r="AL1" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="AM1" t="s">
-        <v>116</v>
+        <v>81</v>
       </c>
       <c r="AN1" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="AO1" t="s">
+        <v>128</v>
+      </c>
+      <c r="AP1" t="s">
+        <v>85</v>
+      </c>
+      <c r="AQ1" t="s">
+        <v>129</v>
+      </c>
+      <c r="AR1" t="s">
+        <v>130</v>
+      </c>
+      <c r="AS1" t="s">
+        <v>131</v>
+      </c>
+      <c r="AT1" t="s">
+        <v>132</v>
+      </c>
+      <c r="AU1" t="s">
+        <v>133</v>
+      </c>
+      <c r="AV1" t="s">
+        <v>134</v>
+      </c>
+      <c r="AW1" t="s">
         <v>118</v>
       </c>
-      <c r="AP1" t="s">
-        <v>119</v>
-      </c>
-      <c r="AQ1" t="s">
-        <v>120</v>
-      </c>
-      <c r="AR1" t="s">
-        <v>121</v>
-      </c>
-      <c r="AS1" t="s">
-        <v>122</v>
-      </c>
-      <c r="AT1" t="s">
-        <v>123</v>
-      </c>
-      <c r="AU1" t="s">
-        <v>124</v>
-      </c>
-      <c r="AV1" t="s">
-        <v>125</v>
-      </c>
-      <c r="AW1" t="s">
-        <v>107</v>
-      </c>
       <c r="AX1" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="AY1" t="s">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="AZ1" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
       <c r="BA1" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="BB1" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="BC1" t="s">
-        <v>131</v>
+        <v>140</v>
       </c>
       <c r="BD1" t="s">
-        <v>40</v>
+        <v>141</v>
       </c>
       <c r="BE1" t="s">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="BF1" t="s">
-        <v>133</v>
+        <v>66</v>
       </c>
       <c r="BG1" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="2" spans="1:59" x14ac:dyDescent="0.3">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="2" spans="1:59" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -3798,262 +3851,262 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:59" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="C3" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="D3" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="E3" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="F3" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G3" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="H3" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="I3" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="J3" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="K3" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="L3" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="M3" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="N3" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="O3" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="P3" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="Q3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="R3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="S3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="T3" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="U3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="V3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="W3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="X3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="Y3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="Z3" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="AA3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="AB3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="AC3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="AD3" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="AE3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="AF3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="AG3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="AH3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="AI3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="AJ3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="AK3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="AL3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="AM3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="AN3" t="s">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="AO3" t="s">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="AP3" t="s">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="AQ3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="AR3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="AS3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="AT3" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="AU3" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="AV3" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="AW3" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="AX3" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="AY3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="AZ3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="BA3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="BB3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="BC3" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="BD3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="BE3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="BF3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="BG3" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="4" spans="1:59" x14ac:dyDescent="0.3">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="4" spans="1:59" x14ac:dyDescent="0.25">
       <c r="M4" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="R4" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="V4" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="W4" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="X4" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="Y4" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="AB4" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="AM4" t="s">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="AQ4" t="s">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="AR4" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="AS4" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="AV4" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="AY4" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="AZ4" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="BA4" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="BB4" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="BD4" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="BE4" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="BF4" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="BG4" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="5" spans="1:59" x14ac:dyDescent="0.3">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="5" spans="1:59" x14ac:dyDescent="0.25">
       <c r="V5" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="Y5" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="AM5" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="AQ5" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="AR5" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="AS5" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -4064,245 +4117,242 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B41"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="36.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="36.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.42578125" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>146</v>
+        <v>155</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>149</v>
+        <v>158</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>155</v>
-      </c>
-      <c r="B8" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>168</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="B12" s="3" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>185</v>
+        <v>194</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>188</v>
+        <v>197</v>
       </c>
     </row>
   </sheetData>

</xml_diff>